<commit_message>
uploading oceanographic data from Romero-romero 2020, plus select data on the North Atlantic.
</commit_message>
<xml_diff>
--- a/Data/Romero-Romero2020.xlsx
+++ b/Data/Romero-Romero2020.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40c9661624813381/Documents/R/North-Pacific-Zooplankton-AA-CSIA-Reanalysis/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40c9661624813381/Documents/R/Mesopelagic_Zooplankton_AA-CSIA_Synthesis/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{F033B481-1499-4CD2-ADEB-2AEC239391CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F836A8B-14B2-4E92-A037-656046FBBE89}"/>
+  <xr:revisionPtr revIDLastSave="209" documentId="13_ncr:1_{F033B481-1499-4CD2-ADEB-2AEC239391CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FADD51C-A69C-4192-B172-96D26177277D}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Romero-Romero2020" sheetId="1" r:id="rId1"/>
+    <sheet name="Romero-Romero2020(wPAP)" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="72">
   <si>
     <t>Site</t>
   </si>
@@ -237,6 +239,18 @@
   </si>
   <si>
     <t>ALOHA W</t>
+  </si>
+  <si>
+    <t>PAP</t>
+  </si>
+  <si>
+    <t>bio.200.night</t>
+  </si>
+  <si>
+    <t>bio.200.day</t>
+  </si>
+  <si>
+    <t>NPP (CAFE)</t>
   </si>
 </sst>
 </file>
@@ -2038,4 +2052,1211 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{912100E8-CAE4-4534-AD07-E4171B3152BB}">
+  <dimension ref="A1:BC9"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="6" max="6" width="19.36328125" customWidth="1"/>
+    <col min="9" max="9" width="9.31640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.54296875" customWidth="1"/>
+    <col min="25" max="25" width="8.2265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.6796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11.6796875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="14" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="9.76953125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="11.6796875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="43" max="44" width="14.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:55" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>71</v>
+      </c>
+      <c r="M1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>14</v>
+      </c>
+      <c r="R1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S1" t="s">
+        <v>16</v>
+      </c>
+      <c r="T1" t="s">
+        <v>17</v>
+      </c>
+      <c r="U1" t="s">
+        <v>18</v>
+      </c>
+      <c r="V1" t="s">
+        <v>19</v>
+      </c>
+      <c r="W1" t="s">
+        <v>20</v>
+      </c>
+      <c r="X1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>46</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>48</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:55" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>155</v>
+      </c>
+      <c r="D2">
+        <v>150</v>
+      </c>
+      <c r="E2">
+        <v>510</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J2">
+        <v>12</v>
+      </c>
+      <c r="K2">
+        <v>44</v>
+      </c>
+      <c r="L2">
+        <f>434/12</f>
+        <v>36.166666666666664</v>
+      </c>
+      <c r="M2" t="s">
+        <v>52</v>
+      </c>
+      <c r="N2" t="s">
+        <v>52</v>
+      </c>
+      <c r="O2">
+        <v>166</v>
+      </c>
+      <c r="P2">
+        <v>120</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>52</v>
+      </c>
+      <c r="R2" t="s">
+        <v>52</v>
+      </c>
+      <c r="S2">
+        <v>353.64</v>
+      </c>
+      <c r="T2">
+        <v>453</v>
+      </c>
+      <c r="U2">
+        <v>287</v>
+      </c>
+      <c r="V2">
+        <v>187</v>
+      </c>
+      <c r="W2" t="s">
+        <v>52</v>
+      </c>
+      <c r="X2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y2">
+        <v>510.37999999999994</v>
+      </c>
+      <c r="Z2">
+        <v>0.36975000000000002</v>
+      </c>
+      <c r="AA2">
+        <v>133.04087717690399</v>
+      </c>
+      <c r="AB2">
+        <v>1037.5</v>
+      </c>
+      <c r="AC2">
+        <v>440</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
+        <v>1.17104397705545E-2</v>
+      </c>
+      <c r="AG2">
+        <v>8.4837476099426396E-3</v>
+      </c>
+      <c r="AH2">
+        <v>3.0525631474624202E-3</v>
+      </c>
+      <c r="AI2">
+        <v>2.38049713193117E-2</v>
+      </c>
+      <c r="AJ2">
+        <v>2.38049713193117E-2</v>
+      </c>
+      <c r="AK2">
+        <v>-20.2285</v>
+      </c>
+      <c r="AL2">
+        <v>34.938000000000002</v>
+      </c>
+      <c r="AM2">
+        <v>1.8381000000000101</v>
+      </c>
+      <c r="AN2">
+        <v>25</v>
+      </c>
+      <c r="AO2">
+        <v>63</v>
+      </c>
+      <c r="AP2">
+        <v>6.9000000000000006E-2</v>
+      </c>
+      <c r="AQ2">
+        <v>0.85337669999999999</v>
+      </c>
+      <c r="AR2">
+        <v>1.0849169999999999</v>
+      </c>
+      <c r="AS2">
+        <v>0.93</v>
+      </c>
+      <c r="AT2">
+        <v>0.91</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AV2">
+        <v>0.78</v>
+      </c>
+      <c r="AW2">
+        <v>0.9</v>
+      </c>
+      <c r="AX2">
+        <v>0.93</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ2">
+        <v>0.98399999999999999</v>
+      </c>
+      <c r="BA2">
+        <v>1.9E-2</v>
+      </c>
+      <c r="BB2">
+        <v>0.98399999999999999</v>
+      </c>
+      <c r="BC2">
+        <v>1.9E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:55" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>155</v>
+      </c>
+      <c r="D3">
+        <v>150</v>
+      </c>
+      <c r="E3">
+        <v>492</v>
+      </c>
+      <c r="F3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3">
+        <v>9</v>
+      </c>
+      <c r="I3" t="s">
+        <v>52</v>
+      </c>
+      <c r="J3">
+        <v>9</v>
+      </c>
+      <c r="K3">
+        <v>27</v>
+      </c>
+      <c r="L3">
+        <f>410/12</f>
+        <v>34.166666666666664</v>
+      </c>
+      <c r="M3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N3" t="s">
+        <v>52</v>
+      </c>
+      <c r="O3">
+        <v>161</v>
+      </c>
+      <c r="P3">
+        <v>120</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>52</v>
+      </c>
+      <c r="R3" t="s">
+        <v>52</v>
+      </c>
+      <c r="S3">
+        <v>45.24</v>
+      </c>
+      <c r="T3">
+        <v>145</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>117</v>
+      </c>
+      <c r="W3" t="s">
+        <v>52</v>
+      </c>
+      <c r="X3" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y3">
+        <v>64.739999999999995</v>
+      </c>
+      <c r="Z3">
+        <v>2.76666666666667E-2</v>
+      </c>
+      <c r="AA3">
+        <v>32</v>
+      </c>
+      <c r="AB3">
+        <v>207.5</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>0</v>
+      </c>
+      <c r="AF3">
+        <v>2.4052012383900898E-3</v>
+      </c>
+      <c r="AG3">
+        <v>1.0278637770897801E-3</v>
+      </c>
+      <c r="AH3">
+        <v>1.1888544891640899E-3</v>
+      </c>
+      <c r="AI3">
+        <v>7.7089783281733704E-3</v>
+      </c>
+      <c r="AJ3">
+        <v>7.7089783281733704E-3</v>
+      </c>
+      <c r="AK3">
+        <v>197.62799999999999</v>
+      </c>
+      <c r="AL3">
+        <v>178.17949999999999</v>
+      </c>
+      <c r="AM3">
+        <v>189.8486</v>
+      </c>
+      <c r="AN3">
+        <v>184</v>
+      </c>
+      <c r="AO3">
+        <v>121</v>
+      </c>
+      <c r="AP3">
+        <v>0.112</v>
+      </c>
+      <c r="AQ3">
+        <v>1.1283399999999999</v>
+      </c>
+      <c r="AR3">
+        <v>1.2335229999999999</v>
+      </c>
+      <c r="AS3">
+        <v>0.92</v>
+      </c>
+      <c r="AT3">
+        <v>0.82</v>
+      </c>
+      <c r="AU3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AV3">
+        <v>0.86</v>
+      </c>
+      <c r="AW3">
+        <v>0.92</v>
+      </c>
+      <c r="AX3">
+        <v>0.92</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ3">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="BA3">
+        <v>0.251</v>
+      </c>
+      <c r="BB3">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="BC3">
+        <v>0.251</v>
+      </c>
+    </row>
+    <row r="4" spans="1:55" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4">
+        <v>22.75</v>
+      </c>
+      <c r="C4">
+        <v>158</v>
+      </c>
+      <c r="D4">
+        <v>132</v>
+      </c>
+      <c r="E4">
+        <v>403.5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4">
+        <v>53</v>
+      </c>
+      <c r="I4">
+        <v>53</v>
+      </c>
+      <c r="J4">
+        <v>16</v>
+      </c>
+      <c r="K4">
+        <v>52</v>
+      </c>
+      <c r="L4">
+        <f>369/12</f>
+        <v>30.75</v>
+      </c>
+      <c r="M4">
+        <v>116</v>
+      </c>
+      <c r="N4">
+        <v>152</v>
+      </c>
+      <c r="O4">
+        <v>180</v>
+      </c>
+      <c r="P4">
+        <v>104</v>
+      </c>
+      <c r="Q4">
+        <v>395.56</v>
+      </c>
+      <c r="R4">
+        <v>590</v>
+      </c>
+      <c r="S4">
+        <v>714.4</v>
+      </c>
+      <c r="T4">
+        <v>265</v>
+      </c>
+      <c r="U4">
+        <v>836</v>
+      </c>
+      <c r="V4">
+        <v>121</v>
+      </c>
+      <c r="W4">
+        <v>1870.64</v>
+      </c>
+      <c r="X4">
+        <v>1981</v>
+      </c>
+      <c r="Y4">
+        <v>1250.5</v>
+      </c>
+      <c r="Z4">
+        <v>1.6659999999999999</v>
+      </c>
+      <c r="AA4">
+        <v>94.589610658065595</v>
+      </c>
+      <c r="AB4">
+        <v>1870.64</v>
+      </c>
+      <c r="AC4">
+        <v>1782.5</v>
+      </c>
+      <c r="AD4">
+        <v>3.5916287999999998E-2</v>
+      </c>
+      <c r="AE4">
+        <v>3.8035199999999998E-2</v>
+      </c>
+      <c r="AF4">
+        <v>2.4009599999999999E-2</v>
+      </c>
+      <c r="AG4">
+        <v>3.15779497709682E-2</v>
+      </c>
+      <c r="AH4">
+        <v>1.7928847384248701E-3</v>
+      </c>
+      <c r="AI4">
+        <v>3.5916287999999998E-2</v>
+      </c>
+      <c r="AJ4">
+        <v>3.5916287999999998E-2</v>
+      </c>
+      <c r="AK4">
+        <v>555.04499999999996</v>
+      </c>
+      <c r="AL4">
+        <v>585.44875000000002</v>
+      </c>
+      <c r="AM4">
+        <v>557.47730000000001</v>
+      </c>
+      <c r="AN4">
+        <v>587</v>
+      </c>
+      <c r="AO4">
+        <v>627</v>
+      </c>
+      <c r="AP4">
+        <v>0.46899999999999997</v>
+      </c>
+      <c r="AQ4">
+        <v>1.0665083</v>
+      </c>
+      <c r="AR4">
+        <v>1.979708</v>
+      </c>
+      <c r="AS4">
+        <v>1</v>
+      </c>
+      <c r="AT4">
+        <v>0.94</v>
+      </c>
+      <c r="AU4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AV4">
+        <v>1</v>
+      </c>
+      <c r="AW4">
+        <v>0.89</v>
+      </c>
+      <c r="AX4">
+        <v>0.94</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ4">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="BA4">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="BB4">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="BC4">
+        <v>9.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:55" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5">
+        <v>22.75</v>
+      </c>
+      <c r="C5">
+        <v>158</v>
+      </c>
+      <c r="D5">
+        <v>132</v>
+      </c>
+      <c r="E5">
+        <v>403.5</v>
+      </c>
+      <c r="F5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5">
+        <v>22</v>
+      </c>
+      <c r="I5">
+        <v>22</v>
+      </c>
+      <c r="J5">
+        <v>23</v>
+      </c>
+      <c r="K5">
+        <v>34</v>
+      </c>
+      <c r="L5">
+        <f>486/12</f>
+        <v>40.5</v>
+      </c>
+      <c r="M5">
+        <v>111</v>
+      </c>
+      <c r="N5">
+        <v>152</v>
+      </c>
+      <c r="O5">
+        <v>168</v>
+      </c>
+      <c r="P5">
+        <v>104</v>
+      </c>
+      <c r="Q5">
+        <v>170.48</v>
+      </c>
+      <c r="R5">
+        <v>414</v>
+      </c>
+      <c r="S5">
+        <v>545.04</v>
+      </c>
+      <c r="T5">
+        <v>97</v>
+      </c>
+      <c r="U5">
+        <v>355</v>
+      </c>
+      <c r="V5">
+        <v>23</v>
+      </c>
+      <c r="W5">
+        <v>479.48</v>
+      </c>
+      <c r="X5">
+        <v>890</v>
+      </c>
+      <c r="Y5">
+        <v>1307.24</v>
+      </c>
+      <c r="Z5">
+        <v>1.0915999999999999</v>
+      </c>
+      <c r="AA5">
+        <v>33.582138109417599</v>
+      </c>
+      <c r="AB5">
+        <v>479.48</v>
+      </c>
+      <c r="AC5">
+        <v>914.5</v>
+      </c>
+      <c r="AD5">
+        <v>1.42915052160954E-2</v>
+      </c>
+      <c r="AE5">
+        <v>2.6527570789865899E-2</v>
+      </c>
+      <c r="AF5">
+        <v>3.8963934426229502E-2</v>
+      </c>
+      <c r="AG5">
+        <v>5.0246260069044903E-2</v>
+      </c>
+      <c r="AH5">
+        <v>1.54578311205605E-3</v>
+      </c>
+      <c r="AI5">
+        <v>1.42915052160954E-2</v>
+      </c>
+      <c r="AJ5">
+        <v>1.42915052160954E-2</v>
+      </c>
+      <c r="AK5">
+        <v>341.91416666666697</v>
+      </c>
+      <c r="AL5">
+        <v>386.22833333333301</v>
+      </c>
+      <c r="AM5">
+        <v>345.45929999999998</v>
+      </c>
+      <c r="AN5">
+        <v>380</v>
+      </c>
+      <c r="AO5">
+        <v>325</v>
+      </c>
+      <c r="AP5">
+        <v>0.42899999999999999</v>
+      </c>
+      <c r="AQ5">
+        <v>0.60651109999999997</v>
+      </c>
+      <c r="AR5">
+        <v>1.2279500000000001</v>
+      </c>
+      <c r="AS5">
+        <v>1</v>
+      </c>
+      <c r="AT5">
+        <v>0.9</v>
+      </c>
+      <c r="AU5" t="s">
+        <v>52</v>
+      </c>
+      <c r="AV5">
+        <v>1</v>
+      </c>
+      <c r="AW5">
+        <v>0.9</v>
+      </c>
+      <c r="AX5">
+        <v>0.93</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ5">
+        <v>0.48199999999999998</v>
+      </c>
+      <c r="BA5">
+        <v>0.189</v>
+      </c>
+      <c r="BB5">
+        <v>0.48199999999999998</v>
+      </c>
+      <c r="BC5">
+        <v>0.189</v>
+      </c>
+    </row>
+    <row r="6" spans="1:55" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6">
+        <v>50.1</v>
+      </c>
+      <c r="C6">
+        <v>144</v>
+      </c>
+      <c r="D6">
+        <v>216</v>
+      </c>
+      <c r="E6">
+        <v>239.4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6">
+        <v>13</v>
+      </c>
+      <c r="I6">
+        <v>13</v>
+      </c>
+      <c r="J6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K6" t="s">
+        <v>52</v>
+      </c>
+      <c r="M6">
+        <v>79</v>
+      </c>
+      <c r="N6">
+        <v>118</v>
+      </c>
+      <c r="O6">
+        <v>118</v>
+      </c>
+      <c r="P6">
+        <v>120</v>
+      </c>
+      <c r="Q6">
+        <v>1444</v>
+      </c>
+      <c r="R6">
+        <v>1428</v>
+      </c>
+      <c r="S6">
+        <v>1428</v>
+      </c>
+      <c r="T6">
+        <v>1428</v>
+      </c>
+      <c r="U6">
+        <v>1028</v>
+      </c>
+      <c r="V6">
+        <v>696</v>
+      </c>
+      <c r="W6">
+        <v>3770</v>
+      </c>
+      <c r="X6">
+        <v>1740</v>
+      </c>
+      <c r="Y6">
+        <v>1740</v>
+      </c>
+      <c r="Z6">
+        <v>1.36666666666667</v>
+      </c>
+      <c r="AA6">
+        <v>369.15820155832603</v>
+      </c>
+      <c r="AB6">
+        <v>1740</v>
+      </c>
+      <c r="AC6">
+        <v>1060</v>
+      </c>
+      <c r="AD6">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="AE6">
+        <v>0.133846153846154</v>
+      </c>
+      <c r="AF6">
+        <v>0.133846153846154</v>
+      </c>
+      <c r="AG6">
+        <v>0.133846153846154</v>
+      </c>
+      <c r="AH6">
+        <v>2.8396784735255899E-2</v>
+      </c>
+      <c r="AI6">
+        <v>2.8396784735255899E-2</v>
+      </c>
+      <c r="AJ6">
+        <v>8.1538461538461504E-2</v>
+      </c>
+      <c r="AK6">
+        <v>219.64673716275701</v>
+      </c>
+      <c r="AL6">
+        <v>256.14891625139398</v>
+      </c>
+      <c r="AM6">
+        <v>257.46937903834402</v>
+      </c>
+      <c r="AN6">
+        <v>236</v>
+      </c>
+      <c r="AO6">
+        <v>341</v>
+      </c>
+      <c r="AP6">
+        <v>0.218</v>
+      </c>
+      <c r="AQ6">
+        <v>2.0392412000000002</v>
+      </c>
+      <c r="AR6">
+        <v>2.5760179999999999</v>
+      </c>
+      <c r="AS6">
+        <v>0.94</v>
+      </c>
+      <c r="AT6">
+        <v>0.93</v>
+      </c>
+      <c r="AU6">
+        <v>0.93</v>
+      </c>
+      <c r="AV6">
+        <v>0.93</v>
+      </c>
+      <c r="AW6">
+        <v>0.88</v>
+      </c>
+      <c r="AX6">
+        <v>0.93</v>
+      </c>
+      <c r="AY6" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ6">
+        <v>1</v>
+      </c>
+      <c r="BA6">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="BB6">
+        <v>0.84</v>
+      </c>
+      <c r="BC6">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:55" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7">
+        <v>75</v>
+      </c>
+      <c r="I7">
+        <v>75</v>
+      </c>
+      <c r="J7" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" t="s">
+        <v>52</v>
+      </c>
+      <c r="M7" t="s">
+        <v>52</v>
+      </c>
+      <c r="N7" t="s">
+        <v>52</v>
+      </c>
+      <c r="O7">
+        <f>AVERAGE(65,93,127)</f>
+        <v>95</v>
+      </c>
+      <c r="P7" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>52</v>
+      </c>
+      <c r="R7" t="s">
+        <v>52</v>
+      </c>
+      <c r="S7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T7" t="s">
+        <v>52</v>
+      </c>
+      <c r="U7" t="s">
+        <v>52</v>
+      </c>
+      <c r="V7" t="s">
+        <v>52</v>
+      </c>
+      <c r="W7" t="s">
+        <v>52</v>
+      </c>
+      <c r="X7" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y7">
+        <f>14.2*1000</f>
+        <v>14200</v>
+      </c>
+      <c r="Z7">
+        <v>11</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AN7">
+        <f>(1785+447)-(1002+372)</f>
+        <v>858</v>
+      </c>
+      <c r="AO7">
+        <v>1833</v>
+      </c>
+      <c r="AP7">
+        <v>0.58599999999999997</v>
+      </c>
+      <c r="AQ7">
+        <v>1.9426334999999999</v>
+      </c>
+      <c r="AR7">
+        <v>6.3454199999999998</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AT7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AU7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AV7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AX7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AY7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ7" t="s">
+        <v>52</v>
+      </c>
+      <c r="BA7" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB7" t="s">
+        <v>52</v>
+      </c>
+      <c r="BC7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:55" ht="44.25" customHeight="1" x14ac:dyDescent="0.75"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D48B64BB-2911-49B1-88D3-CD2D0E18C7CA}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>